<commit_message>
docs: cap nhat cong thuc dac ta Tab 2 theo UI moi (3 the KPI chinh)
</commit_message>
<xml_diff>
--- a/result_docs/Dac_Ta_Y_Nghia_Cong_Thuc_Man_Hinh_Bao_Cao_PineDrama.xlsx
+++ b/result_docs/Dac_Ta_Y_Nghia_Cong_Thuc_Man_Hinh_Bao_Cao_PineDrama.xlsx
@@ -1807,7 +1807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" style="17" min="1" max="1"/>
@@ -1833,348 +1833,268 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>I. CÁC CHỈ SỐ HÀNH VI &amp; THỜI LƯỢNG TƯƠNG TÁC NGƯỜI DÙNG (3 THẺ KPI CHÍNH TRÊN UI MỚI)</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="34" customHeight="1" s="17">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>STT</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Vị trí hiển thị trên màn hình</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Tên trường thông tin (Field Name)</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Ví dụ hiển thị thực tế trên giao diện</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Ý nghĩa của trường (Nghiệp vụ &amp; Người dùng)</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Công thức tính toán (Thuật ngữ người dùng / Logic nghiệp vụ)</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>Quy tắc nghiệp vụ &amp; Điều kiện áp dụng (Business Rules)</t>
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Thẻ thứ 1 (Bên trái) - Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TỶ LỆ GIỮ CHÂN NGƯỜI DÙNG (Retention Rate)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>58.4% (▲ +4.2% so với kỳ trước)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Đo lường năng lực giữ chân khán giả của PineDrama trong kỳ báo cáo: Thể hiện tỷ lệ phần trăm người xem phim có hành vi quay trở lại mở ứng dụng và tiếp tục xem phim trong các ngày tiếp theo của kỳ lọc đã chọn.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1. Công thức chỉ số chính (%):
+Tỷ lệ giữ chân người dùng (%) = (Số lượng người dùng quay lại / Tổng số người dùng Active trong kỳ) × 100%
+• Mẫu số: Số Unique Users có ít nhất 1 phiên xem phim trong kỳ lọc.
+• Tử số: Số Unique Users có phát sinh xem phim ở ít nhất 2 ngày khác nhau trở lên trong kỳ lọc.
+* Trường hợp lọc 1 ngày (D-1): Áp dụng chuẩn D1 Retention: Tỷ lệ D1 (%) = (Số User mới ngày D0 mở lại app ngày D+1 / Tổng User mới ngày D0) × 100%
+2. Công thức biến động so với kỳ trước:
+Biến động (%) = Tỷ lệ giữ chân kỳ này (%) - Tỷ lệ giữ chân kỳ trước liền kề (%) (Điểm phần trăm)
+• Ví dụ: Kỳ này (10/08 - 20/08: 11 ngày) đạt 58.4%, kỳ liền kề trước đó đạt 54.2% -&gt; Biến động: +4.2%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>• Quy tắc màu sắc: Tỷ lệ &gt;= 50% hiển thị màu xanh lá neon #00e676 (Mức Tốt / Xuất sắc); 40% &lt;= Tỷ lệ &lt; 50% hiển thị màu vàng/cam (Trung bình); Tỷ lệ &lt; 40% hiển thị màu đỏ (Cảnh báo).
+• Quy tắc biến động: Tăng hiển thị icon ▲ dấu + màu xanh lá; Giảm hiển thị icon ▼ dấu - màu đỏ.
+• Điều kiện: Chốt số liệu sau khi kết thúc 23:59:59 của ngày cuối cùng trong kỳ. Làm tròn 1 chữ số thập phân (58.4%).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="17">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>I. CÁC CHỈ SỐ GIỮ CHÂN NGƯỜI DÙNG THEO THỜI GIAN (USER RETENTION COHORT)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
-      <c r="F5" s="14" t="n"/>
-      <c r="G5" s="15" t="n"/>
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Thẻ thứ 2 (Ở giữa) - Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>THỜI GIAN XEM TRUNG BÌNH (Average Daily Watch Time)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>48.5 Phút / Ngày (▲ +6.5 phút so với kỳ trước)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Khắc họa mức độ nghiện phim và tiêu thụ nội dung hàng ngày của khán giả: Trung bình mỗi ngày một khán giả xem phim dành ra bao nhiêu phút trên PineDrama. Chỉ số này càng cao chứng tỏ khán giả có thói quen xem liên tục nhiều tập phim (cày phim - Binge-watching).</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1. Công thức chỉ số chính (Phút/Ngày):
+Thời gian xem TB (Phút/Ngày) = (Tổng số phút xem video của tất cả người dùng trong kỳ) / (Tổng số lượt User-Day hoạt động trong kỳ)
+• Tổng số phút xem: Tổng thời lượng phát video thực tế của tất cả khán giả trong kỳ (phút).
+• Tổng số lượt User-Day: Tổng cộng số ngày có xem phim của từng người dùng trong kỳ.
+• Ví dụ: Kỳ lọc 11 ngày có tổng 6,052,800 phút xem và 124,800 lượt User-Day -&gt; TB = 6,052,800 / 124,800 = 48.5 Phút/Ngày.
+2. Công thức biến động so với kỳ trước:
+Biến động (phút) = Thời gian xem TB kỳ này - Thời gian xem TB kỳ trước liền kề
+• Ví dụ: Kỳ này 48.5 phút/ngày, kỳ trước 42.0 phút/ngày -&gt; Biến động: +6.5 phút.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>• Chuẩn ngành phim ngắn: &gt;= 40 Phút/Ngày là mức Rất cao; 25 - 40 Phút/Ngày là Khá/Ổn định; &lt; 25 Phút/Ngày là Thấp.
+• Chống treo máy: Phiên xem liên tục không tương tác sau 3 giờ sẽ ngưng tính thời lượng từ phút 181 để tránh sai lệch do ngủ quên/treo máy.
+• Hiển thị: Làm tròn 1 chữ số thập phân, biến động hiển thị màu xanh dương neon #40c4ff.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="175.5" customHeight="1" s="17">
-      <c r="A6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Khối thẻ góc trái trên của Tab 2</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Thẻ thứ 3 (Bên phải) - Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NGƯỜI DÙNG ACTIVE (Active Users in Period)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>124,800 Người (▲ +12.8% so với kỳ trước)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Đo lường quy mô khán giả thực tế tiếp cận và tiêu thụ nội dung trên nền tảng trong khoảng thời gian được lọc. Đây là chỉ số nền tảng quyết định độ lớn của thị phần người xem, sức sống ứng dụng và tiềm năng doanh thu.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1. Công thức chỉ số chính (Người):
+Người dùng Active = COUNT(DISTINCT user_id) trong kỳ lọc đã chọn
+• Điều kiện: Tài khoản hoặc thiết bị có sự kiện xem phim &gt;= 5 giây hoặc hoàn thành ít nhất 1 tập.
+• Khử trùng lặp: Mỗi người dùng chỉ tính 1 lần duy nhất trong toàn kỳ lọc dù xem phim ở nhiều ngày.
+2. Công thức tăng trưởng so với kỳ trước:
+Tăng trưởng (%) = [(Active kỳ này - Active kỳ trước) / Active kỳ trước] × 100%
+• Ví dụ: Kỳ này 124,800 người, kỳ trước 110,638 người -&gt; Tăng trưởng: +12.8%.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>• Tệp người dùng: Bao gồm cả User có tài khoản và Khách vãng lai (Guest qua Device ID).
+• Hiển thị: Định dạng có dấu phẩy phân cách hàng nghìn kèm chữ "Người" (124,800 Người).
+• Biến động: Tăng trưởng dương hiển thị icon ▲ dấu + màu xanh lá; Giảm hiển thị icon ▼ dấu - màu đỏ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1" s="17">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>II. CÁC CHỈ SỐ PHÂN TÍCH CHUYÊN SÂU (RETENTION COHORT CHI TIẾT - PHỤC VỤ DRILL-DOWN BÁO CÁO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="240" customHeight="1" s="17">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Phân tích Cohort chi tiết</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>D1 Retention (Quay lại sau 1 ngày)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>58.4% (Tốt)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Tỷ lệ người dùng mới cảm thấy thích thú với ứng dụng và quay lại mở app xem tiếp ngay vào ngày hôm sau (D+1).</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>1. Khi lọc 1 ngày (D-1): Tỷ lệ D1 (%) = (Số user trong nhóm D0 quay lại vào ngày D+1 / Tổng user mới nhóm D0) x 100%.
-• Ví dụ: Ngày 10/08 có 10,000 user mới, ngày 11/08 có 5,840 người mở lại app -&gt; D1 = 58.4%.
-2. Khi lọc KHOẢNG NGÀY (VD: 10/08 - 30/08, gồm 20 ngày): Là TRUNG BÌNH CÓ TRỌNG SỐ (không phải cộng tổng %):
-• D1 (Kỳ) = (Tổng User quay lại ngày D+1 của cả 20 nhóm / Tổng User mới của cả 20 nhóm) x 100%.
-• Ví dụ: Cả 20 ngày có 200,000 user mới, tổng số người quay lại D+1 của các ngày là 113,600 người -&gt; D1 trung bình = (113,600 / 200,000) x 100% = 56.8%.</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>• D1 chỉ chốt số trọn vẹn khi ngày hiện tại tối thiểu là ngày hôm sau của ngày cuối cùng trong kỳ lọc.
-• Chuẩn ngành phim ngắn: D1 &gt; 50% là mức xuất sắc (gắn nhãn xanh lá 'Tốt'). Dưới 40% là cảnh báo nội dung chưa đủ cuốn hút.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="128" customHeight="1" s="17">
-      <c r="A7" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Khối thẻ góc trái dưới của Tab 2</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>58.4%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Tỷ lệ người dùng mới có ấn tượng tích cực và quay lại mở app xem tiếp ngay vào ngày hôm sau (D+1).</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1. Lọc 1 ngày: Tỷ lệ D1 (%) = (Số user mới ngày D0 mở lại app ngày D+1 / Tổng user mới ngày D0) x 100%
+2. Lọc khoảng ngày: Trung bình có trọng số của các ngày đã hoàn thành chu kỳ D+1.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>• Chuẩn ngành phim ngắn: &gt;= 50% là Tốt/Xuất sắc; &lt; 40% là cảnh báo nội dung tập đầu chưa đủ cuốn hút. Chỉ chốt số liệu khi qua ngày D+1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="67.5" customHeight="1" s="17">
+      <c r="A9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Phân tích Cohort chi tiết</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>D7 Retention (Quay lại sau 7 ngày)</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>34.8%</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>Đo lường thói quen xem phim hàng tuần của người dùng sau 7 ngày trải nghiệm (D+7).</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>1. Khi lọc 1 ngày: Tỷ lệ D7 (%) = (Số user trong nhóm D0 còn quay lại vào ngày thứ 7 / Tổng user mới nhóm D0) x 100%.
-2. Khi lọc KHOẢNG NGÀY: Là TRUNG BÌNH CÓ TRỌNG SỐ của các nhóm người dùng trong kỳ đã hoàn thành chu kỳ 7 ngày (D0 + 7 ngày).</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>• Chu kỳ 7 ngày trượt (Rolling 7 Days) tính từ ngày D0 cộng thêm 7 ngày.
-• Nếu ngày được chọn chưa trôi qua đủ 7 ngày so với hiện tại -&gt; Hiển thị dấu gạch ngang '--' (Chờ đủ 7 ngày), tuyệt đối không để 0%.
-• Mức chuẩn tốt của ứng dụng phim ngắn đạt từ 30% đến 40%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="240" customHeight="1" s="17">
-      <c r="A8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Khối thẻ góc phải trên của Tab 2</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Đo lường thói quen xem phim hàng tuần của khán giả mới sau 1 tuần trải nghiệm ứng dụng (D+7).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1. Lọc 1 ngày: Tỷ lệ D7 (%) = (Số user mới ngày D0 còn quay lại ngày D+7 / Tổng user mới ngày D0) x 100%
+2. Lọc khoảng ngày: Trung bình có trọng số của các nhóm user đã đủ 7 ngày tuổi.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>• Chuẩn ngành: Đạt từ 30% đến 40% là Tốt. Những ngày chưa đủ 7 ngày tuổi không đưa vào mẫu số.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="17">
+      <c r="A10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Phân tích Cohort chi tiết</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>D30 Retention (Quay lại sau 30 ngày)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>21.2%</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Tỷ lệ khán giả trung thành còn gắn bó với ứng dụng sau 1 tháng sử dụng (D+30). Đây là tệp người dùng cốt lõi mang lại giá trị vòng đời (LTV) lâu dài.</t>
-        </is>
-      </c>
-      <c r="F8" s="24" t="inlineStr">
-        <is>
-          <t>1. BẢN CHẤT CHU KỲ 30 NGÀY (VẮT SANG THÁNG TIẾP THEO):
-• D30 là chu kỳ 30 ngày trượt tính từ ngày người dùng cài app (D0) VẮT SANG THÁNG TIẾP THEO (D0 + 30 ngày), KHÔNG PHẢI chỉ tính trong 30 ngày của cùng một tháng dương lịch:
-  + Khách vào ngày 05/08 -&gt; Mốc D30 chốt sổ vào ngày 04/09 (tháng sau).
-  + Khách vào ngày 15/08 -&gt; Mốc D30 chốt sổ vào ngày 14/09 (tháng sau).
-  + Khách vào ngày 30/08 -&gt; Mốc D30 chốt sổ vào ngày 29/09 (tháng sau).
-2. GIẢI THÍCH RÕ RÀNG KHI LỌC KHOẢNG NGÀY (VÍ DỤ: 10/08 - 30/08, DÀI 20 NGÀY):
-• Sự khác biệt giữa 2 khái niệm:
-  - Dải ngày lọc (10/08 - 30/08): Là KHOẢNG NGÀY SINH RA USER MỚI (ngày khách cài App D0).
-  - Chỉ số D30: Là số % user đó CÒN QUAY LẠI VÀO NGÀY THỨ 30 CỦA HỌ (rơi vào tháng 9).
-• Ví dụ minh họa thực tế khi mở màn hình xem báo cáo:
-  + Trường hợp 1: Nếu hôm nay là Tháng 10/2026 mở lọc kỳ 10/08 - 30/08: Vì thời gian thực tế đã qua tháng 9, toàn bộ user sinh ra từ 10/08 đến 30/08 ĐỀU ĐÃ SỐNG ĐỦ 30 NGÀY VÒNG ĐỜI (đã bước qua các ngày chốt sổ 09/09 -&gt; 29/09). Do đó hệ thống tính được D30 trọn vẹn cho cả nhóm!
-  + Công thức tính D30 cả kỳ là TRUNG BÌNH CÓ TRỌNG SỐ:
-    D30 cả kỳ = (Tổng user ngày D+30 còn vào App / Tổng user mới cả 20 ngày) × 100%
-    (Tuyệt đối KHÔNG PHẢI cộng dồn các con số % lại với nhau).
-  + Trường hợp 2: Nếu hôm nay là ngày 31/08/2026 (vừa hết kỳ lọc xem ngay): Trong đời thực chưa có user nào bước sang tháng 9 để đủ 30 ngày tuổi -&gt; Hiển thị '--' (Đang tích lũy chu kỳ).
-  + Trường hợp 3: Nếu hôm nay là ngày 20/09/2026: Khách từ 10/08-20/08 đã đủ 30 ngày; khách từ 21/08-30/08 chưa đủ -&gt; Hệ thống lấy trung bình D30 của những ngày đã đủ 30 ngày (kèm ghi chú *).</t>
-        </is>
-      </c>
-      <c r="G8" s="25" t="inlineStr">
-        <is>
-          <t>• QUY TẮC HIỂN THỊ KHI CHƯA ĐỦ 30 NGÀY:
-  + Tuyệt đối KHÔNG hiển thị '0%' hay lỗi 'NaN' khi chưa đủ thời gian kiểm chứng.
-  + Nếu chưa có ngày nào trong kỳ lọc đủ 30 ngày trôi qua (ví dụ lọc ngày hôm qua D-1, hoặc vừa hết tháng xem ngay) -&gt; Hiển thị dấu gạch ngang '--' (Đang tích lũy chu kỳ) với màu xám mờ.
-  + Nếu một phần ngày đã đủ 30 ngày, một phần chưa đủ (ví dụ đang ở giữa tháng 9 xem kỳ tháng 8) -&gt; Hệ thống tính trung bình D30 trên các nhóm ngày đã hoàn thành chu kỳ (kèm dấu hoa thị * giải thích).
-• Ý NGHĨA KINH DOANH: Chỉ số vàng đo lường độ trung thành và giá trị vòng đời (LTV) lâu dài của người dùng. Giữ chân D30 tốt mới quyết định hiệu quả khi mở rộng quy mô chạy marketing/quảng cáo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="67.5" customHeight="1" s="17">
-      <c r="A9" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Khối thẻ góc phải dưới của Tab 2</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Thời gian xem trung bình mỗi User</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>48.5 Phút / Ngày</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Khắc họa mức độ nghiện phim của khán giả: Trung bình mỗi ngày một người dùng dành ra bao nhiêu phút để xem phim trên PineDrama.</t>
-        </is>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>Thời gian xem TB mỗi User = Tổng số phút xem video của tất cả người dùng trong ngày chia cho Tổng số người dùng hoạt động trong ngày.
-• Ví dụ: Tổng thời gian xem 6,052,800 phút / 124,800 Active Users = 48.5 phút/người/ngày.</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>Mức trung bình &gt; 40 phút/ngày chứng tỏ khán giả có thói quen xem liên tục nhiều tập phim (cày phim - Binge-watching).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16.5" customHeight="1" s="17">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>II. CÁC CHỈ SỐ PHÂN TÍCH HÀNH VI MỞ RỘNG (DÀNH CHO BÁO CÁO CHI TIẾT)</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="15" t="n"/>
-    </row>
-    <row r="11" ht="48" customHeight="1" s="17">
-      <c r="A11" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Chỉ số mở rộng quy mô</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Số người dùng hoạt động hàng ngày (DAU)</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>124,800 Users</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Quy mô lượng khán giả thực tế truy cập và sử dụng ứng dụng mỗi ngày.</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>Tổng số tài khoản hoặc thiết bị duy nhất có mở ứng dụng và phát sinh tương tác trong ngày.</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>Mỗi người dù mở app nhiều lần trong ngày thì cũng chỉ được tính là 1 DAU duy nhất.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1" s="17">
-      <c r="A12" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Chỉ số mở rộng tăng trưởng</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Số người dùng cài mới (New Users)</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>15,200 Người dùng mới</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Tốc độ thu hút khán giả mới cài đặt hoặc đăng ký tài khoản lần đầu trên nền tảng trong kỳ báo cáo.</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Tổng số thiết bị lần đầu cài đặt ứng dụng hoặc tài khoản mới tạo trong khoảng thời gian lọc.</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Loại trừ các trường hợp gỡ app rồi cài đặt lại trên cùng một thiết bị.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1" s="17">
-      <c r="A13" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Chỉ số mở rộng tương tác</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Số phiên mở app trung bình (Sessions per User)</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>3.8 Phiên / Ngày</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>Khán giả có thói quen mở ứng dụng bao nhiêu lần trong một ngày (các khung giờ rảnh như nghỉ trưa, đi xe bus, buổi tối).</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>Số phiên trung bình = Tổng số lần mở ứng dụng của tất cả người dùng / Tổng số người dùng hoạt động trong ngày.</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>Mỗi phiên được tính từ lúc mở app đến lúc tắt hoặc không tương tác quá 30 phút.</t>
-        </is>
-      </c>
-    </row>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Tỷ lệ khán giả trung thành cốt lõi còn gắn bó với ứng dụng sau 1 tháng sử dụng (D+30).</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1. Lọc 1 ngày: Tỷ lệ D30 (%) = (Số user mới ngày D0 mở lại app ngày D+30 / Tổng user mới ngày D0) x 100%
+2. Lọc khoảng ngày: Trung bình có trọng số của các nhóm user đã đủ 30 ngày tuổi.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>• Chuẩn ngành: &gt;= 20% là xuất sắc. Nếu chưa đủ 30 ngày hiển thị dấu gạch ngang "--" (Đang tích lũy chu kỳ), không để 0% hoặc NaN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" s="17"/>
+    <row r="12" ht="48" customHeight="1" s="17"/>
+    <row r="13" ht="48" customHeight="1" s="17"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>